<commit_message>
Changed the name of the files and fixed the Dark Mode and export html
</commit_message>
<xml_diff>
--- a/DadsProjects.xlsx
+++ b/DadsProjects.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Python\DadsProjects\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48D98BE4-F728-4850-A599-D37695E1292F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{569BCF86-DB34-4A15-89F1-93CF50EF25C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -54,21 +54,12 @@
     <t>Easter 2025_1.jpg</t>
   </si>
   <si>
-    <t>Fête des Mères de mon père 2023.jpg</t>
-  </si>
-  <si>
     <t>Holloween 2024_1.jpg</t>
   </si>
   <si>
     <t>Holloween_2025.jpg</t>
   </si>
   <si>
-    <t>Maquette-Paques de mon père 2023_2.jpg</t>
-  </si>
-  <si>
-    <t>Noël des campeurs 2024_1.jpg</t>
-  </si>
-  <si>
     <t>Paques_2026.jpg</t>
   </si>
   <si>
@@ -112,6 +103,15 @@
   </si>
   <si>
     <t>Valentine's Day</t>
+  </si>
+  <si>
+    <t>Mothers_Day 2023.jpg</t>
+  </si>
+  <si>
+    <t>Christmas_For_The_Campers 2024_1.jpg</t>
+  </si>
+  <si>
+    <t>Fathers_Day 2023_2.jpg</t>
   </si>
 </sst>
 </file>
@@ -457,7 +457,7 @@
         <v>2026</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -468,7 +468,7 @@
         <v>2023</v>
       </c>
       <c r="C3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -479,7 +479,7 @@
         <v>2024</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -490,7 +490,7 @@
         <v>2024</v>
       </c>
       <c r="C5" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -501,128 +501,128 @@
         <v>2025</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="B7">
         <v>2023</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B8">
         <v>2024</v>
       </c>
       <c r="C8" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B9">
         <v>2025</v>
       </c>
       <c r="C9" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="B10">
         <v>2023</v>
       </c>
       <c r="C10" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="B11">
         <v>2024</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B12">
         <v>2026</v>
       </c>
       <c r="C12" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B13">
         <v>2025</v>
       </c>
       <c r="C13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B14">
         <v>2024</v>
       </c>
       <c r="C14" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B15">
         <v>2025</v>
       </c>
       <c r="C15" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B16">
         <v>2025</v>
       </c>
       <c r="C16" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B17">
         <v>2026</v>
       </c>
       <c r="C17" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>